<commit_message>
Initial Playwright TypeScript project (clean, no secrets)
</commit_message>
<xml_diff>
--- a/testdata/bulckupload0.xlsx
+++ b/testdata/bulckupload0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasikani\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CCEC10-A616-4A36-A537-78668CE0A34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9F5B512-497D-4F39-8806-21DEE8FDD30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -93,66 +93,6 @@
     <t>LastName</t>
   </si>
   <si>
-    <t>adhilingam18+f3t1@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t2@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t3@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t4@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t5@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t6@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t7@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t8@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t9@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t10@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t11@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t12@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t13@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t14@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t15@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t16@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t17@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t18@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t19@gmail.com</t>
-  </si>
-  <si>
-    <t>adhilingam18+f3t20@gmail.com</t>
-  </si>
-  <si>
     <t>Leonardo</t>
   </si>
   <si>
@@ -163,6 +103,9 @@
   </si>
   <si>
     <t>Pitt</t>
+  </si>
+  <si>
+    <t>Tom</t>
   </si>
   <si>
     <t>Hanks</t>
@@ -267,7 +210,64 @@
     <t>Phoenix</t>
   </si>
   <si>
-    <t>Tomq</t>
+    <t>adhilingam18+f3t21@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t22@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t23@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t24@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t25@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t26@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t27@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t28@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t29@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t30@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t31@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t32@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t33@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t34@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t35@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t36@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t37@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t38@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t39@gmail.com</t>
+  </si>
+  <si>
+    <t>adhilingam18+f3t40@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -849,13 +849,13 @@
     </row>
     <row r="3" spans="1:13" ht="14" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -885,13 +885,13 @@
     </row>
     <row r="4" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4">
@@ -921,13 +921,13 @@
     </row>
     <row r="5" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4">
@@ -957,13 +957,13 @@
     </row>
     <row r="6" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4">
@@ -993,13 +993,13 @@
     </row>
     <row r="7" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4">
@@ -1029,13 +1029,13 @@
     </row>
     <row r="8" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4">
@@ -1065,13 +1065,13 @@
     </row>
     <row r="9" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4">
@@ -1101,13 +1101,13 @@
     </row>
     <row r="10" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4">
@@ -1137,13 +1137,13 @@
     </row>
     <row r="11" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4">
@@ -1173,13 +1173,13 @@
     </row>
     <row r="12" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4">
@@ -1209,13 +1209,13 @@
     </row>
     <row r="13" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4">
@@ -1245,13 +1245,13 @@
     </row>
     <row r="14" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4">
@@ -1281,13 +1281,13 @@
     </row>
     <row r="15" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4">
@@ -1317,13 +1317,13 @@
     </row>
     <row r="16" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4">
@@ -1353,13 +1353,13 @@
     </row>
     <row r="17" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4">
@@ -1389,13 +1389,13 @@
     </row>
     <row r="18" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4">
@@ -1425,13 +1425,13 @@
     </row>
     <row r="19" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4">
@@ -1461,13 +1461,13 @@
     </row>
     <row r="20" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4">
@@ -1497,13 +1497,13 @@
     </row>
     <row r="21" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>79</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4">
@@ -1533,13 +1533,13 @@
     </row>
     <row r="22" spans="1:13" ht="14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4">

</xml_diff>